<commit_message>
Add Volvo, Land Rover and Ford transponder DBs; extra Lexus OEM keys
- Volvo: Korean-spec 447MHz smart key 31300259 (P1), P2/P3/SPA generations
- Land Rover: part numbers limited to confirmed 433/434MHz keys, EWS/ID46 transition rows
- Ford: 434MHz export keys and frequency-free transponder/emergency keys only; Korean sales years
- Lexus: IS card keys, LS460 433MHz smart keys from auto-keys.eu

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GdWs29tcwv2723Uq4P5rH7
</commit_message>
<xml_diff>
--- a/렉서스_models.xlsx
+++ b/렉서스_models.xlsx
@@ -2046,7 +2046,7 @@
       </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키,카드키</t>
         </is>
       </c>
       <c r="I22" s="9" t="inlineStr">
@@ -2059,10 +2059,14 @@
           <t>TOY48</t>
         </is>
       </c>
-      <c r="K22" s="9" t="inlineStr"/>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>89904-50480[해외 공용 품번], 89904-50481[해외 공용 품번], 89904-53131[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="L22" s="9" t="inlineStr">
         <is>
-          <t>89904-53361[해외 공용 품번]</t>
+          <t>89904-53361[해외 공용 품번], 89904-53321[해외 공용 품번], 89904-53322[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr"/>
@@ -2073,7 +2077,7 @@
       </c>
       <c r="O22" s="9" t="inlineStr">
         <is>
-          <t>transpondery(IS 2009–2013 Texas G DST80), abkeys(순정 89904-53361 433MHz P1 98 IS250 2007-2013 유럽·중동)</t>
+          <t>transpondery(IS 2009–2013 Texas G DST80, 카드키 블랭크 69515-50270→69515-30350), abkeys(순정 89904-53361 433MHz P1 98 IS250 2007-2013 유럽·중동), auto-keys.eu(순정 89904-53321·53322 433MHz P1 98, IS250·350 스마트 카드 89904-53131·50480·50481 433MHz)</t>
         </is>
       </c>
       <c r="P22" s="9" t="inlineStr"/>
@@ -2116,7 +2120,7 @@
       </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키,카드키</t>
         </is>
       </c>
       <c r="I23" s="9" t="inlineStr">
@@ -2129,10 +2133,14 @@
           <t>TOY48</t>
         </is>
       </c>
-      <c r="K23" s="9" t="inlineStr"/>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>89904-50480[해외 공용 품번], 89904-50481[해외 공용 품번], 89904-53131[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>89904-53361[해외 공용 품번]</t>
+          <t>89904-53361[해외 공용 품번], 89904-53321[해외 공용 품번], 89904-53322[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr"/>
@@ -2143,7 +2151,7 @@
       </c>
       <c r="O23" s="9" t="inlineStr">
         <is>
-          <t>transpondery(IS 2009–2013 Texas G DST80), abkeys(순정 89904-53361 433MHz P1 98 IS250 2007-2013 유럽·중동)</t>
+          <t>transpondery(IS 2009–2013 Texas G DST80, 카드키 블랭크 69515-50270→69515-30350), abkeys(순정 89904-53361 433MHz P1 98 IS250 2007-2013 유럽·중동), auto-keys.eu(순정 89904-53321·53322 433MHz P1 98, IS250·350 스마트 카드 89904-53131·50480·50481 433MHz)</t>
         </is>
       </c>
       <c r="P23" s="9" t="inlineStr"/>
@@ -2186,7 +2194,7 @@
       </c>
       <c r="H24" s="9" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키,카드키</t>
         </is>
       </c>
       <c r="I24" s="9" t="inlineStr">
@@ -2199,10 +2207,14 @@
           <t>TOY48</t>
         </is>
       </c>
-      <c r="K24" s="9" t="inlineStr"/>
+      <c r="K24" s="9" t="inlineStr">
+        <is>
+          <t>89904-50480[해외 공용 품번], 89904-50481[해외 공용 품번], 89904-53131[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>89904-53361[해외 공용 품번]</t>
+          <t>89904-53361[해외 공용 품번], 89904-53321[해외 공용 품번], 89904-53322[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr"/>
@@ -2213,7 +2225,7 @@
       </c>
       <c r="O24" s="9" t="inlineStr">
         <is>
-          <t>transpondery(IS 2009–2013 Texas G DST80), abkeys(순정 89904-53361 433MHz P1 98 IS250 2007-2013 유럽·중동)</t>
+          <t>transpondery(IS 2009–2013 Texas G DST80, 카드키 블랭크 69515-50270→69515-30350), abkeys(순정 89904-53361 433MHz P1 98 IS250 2007-2013 유럽·중동), auto-keys.eu(순정 89904-53321·53322 433MHz P1 98, IS250·350 스마트 카드 89904-53131·50480·50481 433MHz)</t>
         </is>
       </c>
       <c r="P24" s="9" t="inlineStr"/>
@@ -2256,7 +2268,7 @@
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키,카드키</t>
         </is>
       </c>
       <c r="I25" s="9" t="inlineStr">
@@ -2269,10 +2281,14 @@
           <t>TOY48</t>
         </is>
       </c>
-      <c r="K25" s="9" t="inlineStr"/>
+      <c r="K25" s="9" t="inlineStr">
+        <is>
+          <t>89904-50480[해외 공용 품번], 89904-50481[해외 공용 품번], 89904-53131[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>89904-53361[해외 공용 품번]</t>
+          <t>89904-53361[해외 공용 품번], 89904-53321[해외 공용 품번], 89904-53322[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr"/>
@@ -2283,7 +2299,7 @@
       </c>
       <c r="O25" s="9" t="inlineStr">
         <is>
-          <t>transpondery(IS 2009–2013 Texas G DST80), abkeys(순정 89904-53361 433MHz P1 98 IS250 2007-2013 유럽·중동)</t>
+          <t>transpondery(IS 2009–2013 Texas G DST80, 카드키 블랭크 69515-50270→69515-30350), abkeys(순정 89904-53361 433MHz P1 98 IS250 2007-2013 유럽·중동), auto-keys.eu(순정 89904-53321·53322 433MHz P1 98, IS250·350 스마트 카드 89904-53131·50480·50481 433MHz)</t>
         </is>
       </c>
       <c r="P25" s="9" t="inlineStr"/>
@@ -2326,7 +2342,7 @@
       </c>
       <c r="H26" s="9" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키,카드키</t>
         </is>
       </c>
       <c r="I26" s="9" t="inlineStr">
@@ -2339,10 +2355,14 @@
           <t>TOY48</t>
         </is>
       </c>
-      <c r="K26" s="9" t="inlineStr"/>
+      <c r="K26" s="9" t="inlineStr">
+        <is>
+          <t>89904-50480[해외 공용 품번], 89904-50481[해외 공용 품번], 89904-53131[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>89904-53361[해외 공용 품번]</t>
+          <t>89904-53361[해외 공용 품번], 89904-53321[해외 공용 품번], 89904-53322[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr"/>
@@ -2353,7 +2373,7 @@
       </c>
       <c r="O26" s="9" t="inlineStr">
         <is>
-          <t>transpondery(IS 2009–2013 Texas G DST80), abkeys(순정 89904-53361 433MHz P1 98 IS250 2007-2013 유럽·중동)</t>
+          <t>transpondery(IS 2009–2013 Texas G DST80, 카드키 블랭크 69515-50270→69515-30350), abkeys(순정 89904-53361 433MHz P1 98 IS250 2007-2013 유럽·중동), auto-keys.eu(순정 89904-53321·53322 433MHz P1 98, IS250·350 스마트 카드 89904-53131·50480·50481 433MHz)</t>
         </is>
       </c>
       <c r="P26" s="9" t="inlineStr"/>
@@ -6958,7 +6978,7 @@
       <c r="K94" s="9" t="inlineStr"/>
       <c r="L94" s="9" t="inlineStr">
         <is>
-          <t>89904-30320[해외 공용 품번], 89904-30322[해외 공용 품번]</t>
+          <t>89904-30322[해외 공용 품번], 89904-30323[해외 공용 품번], 89904-50561[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M94" s="9" t="inlineStr"/>
@@ -6969,7 +6989,7 @@
       </c>
       <c r="O94" s="9" t="inlineStr">
         <is>
-          <t>transpondery(LS 460 2007–2008 TMS37126 DST40 Page1 94, 비상키 69515-50260), abkeys(89904-30320·30322 ES GS IS LS 2006+ 433MHz)</t>
+          <t>transpondery(LS 460 2007–2008 TMS37126 DST40 Page1 94, 비상키 69515-50260), auto-keys.eu(순정 89904-30322·30323 433MHz ES350·GS·IS·LS460, LS460 2008 89904-50561 433MHz Tiris 4D)</t>
         </is>
       </c>
       <c r="P94" s="9" t="inlineStr"/>
@@ -7028,7 +7048,7 @@
       <c r="K95" s="9" t="inlineStr"/>
       <c r="L95" s="9" t="inlineStr">
         <is>
-          <t>89904-30320[해외 공용 품번], 89904-30322[해외 공용 품번]</t>
+          <t>89904-30322[해외 공용 품번], 89904-30323[해외 공용 품번], 89904-50561[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M95" s="9" t="inlineStr"/>
@@ -7039,7 +7059,7 @@
       </c>
       <c r="O95" s="9" t="inlineStr">
         <is>
-          <t>transpondery(LS 460 2007–2008 TMS37126 DST40 Page1 94, 비상키 69515-50260), abkeys(89904-30320·30322 ES GS IS LS 2006+ 433MHz)</t>
+          <t>transpondery(LS 460 2007–2008 TMS37126 DST40 Page1 94, 비상키 69515-50260), auto-keys.eu(순정 89904-30322·30323 433MHz ES350·GS·IS·LS460, LS460 2008 89904-50561 433MHz Tiris 4D)</t>
         </is>
       </c>
       <c r="P95" s="9" t="inlineStr"/>
@@ -7098,7 +7118,7 @@
       <c r="K96" s="9" t="inlineStr"/>
       <c r="L96" s="9" t="inlineStr">
         <is>
-          <t>89904-30320[해외 공용 품번], 89904-30322[해외 공용 품번]</t>
+          <t>89904-30322[해외 공용 품번], 89904-30323[해외 공용 품번], 89904-50561[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M96" s="9" t="inlineStr"/>
@@ -7109,7 +7129,7 @@
       </c>
       <c r="O96" s="9" t="inlineStr">
         <is>
-          <t>transpondery(LS 460 2007–2008 TMS37126 DST40 Page1 94, 비상키 69515-50260), abkeys(89904-30320·30322 ES GS IS LS 2006+ 433MHz)</t>
+          <t>transpondery(LS 460 2007–2008 TMS37126 DST40 Page1 94, 비상키 69515-50260), auto-keys.eu(순정 89904-30322·30323 433MHz ES350·GS·IS·LS460, LS460 2008 89904-50561 433MHz Tiris 4D)</t>
         </is>
       </c>
       <c r="P96" s="9" t="inlineStr"/>
@@ -7166,7 +7186,11 @@
         </is>
       </c>
       <c r="K97" s="9" t="inlineStr"/>
-      <c r="L97" s="9" t="inlineStr"/>
+      <c r="L97" s="9" t="inlineStr">
+        <is>
+          <t>89904-50L00[해외 공용 품번], 89904-50L01[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="M97" s="9" t="inlineStr"/>
       <c r="N97" s="9" t="inlineStr">
         <is>
@@ -7175,7 +7199,7 @@
       </c>
       <c r="O97" s="9" t="inlineStr">
         <is>
-          <t>transpondery(LS 460·600h 2009–2012 Texas G DST80 — 433MHz 품번 자료 없음)</t>
+          <t>transpondery(LS 460·600h 2009–2012 Texas G DST80), auto-keys.eu(순정 LS 460 89904-50L00·50L01 433MHz P1 98)</t>
         </is>
       </c>
       <c r="P97" s="9" t="inlineStr"/>
@@ -7232,7 +7256,11 @@
         </is>
       </c>
       <c r="K98" s="9" t="inlineStr"/>
-      <c r="L98" s="9" t="inlineStr"/>
+      <c r="L98" s="9" t="inlineStr">
+        <is>
+          <t>89904-50L00[해외 공용 품번], 89904-50L01[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="M98" s="9" t="inlineStr"/>
       <c r="N98" s="9" t="inlineStr">
         <is>
@@ -7241,7 +7269,7 @@
       </c>
       <c r="O98" s="9" t="inlineStr">
         <is>
-          <t>transpondery(LS 460·600h 2009–2012 Texas G DST80 — 433MHz 품번 자료 없음)</t>
+          <t>transpondery(LS 460·600h 2009–2012 Texas G DST80), auto-keys.eu(순정 LS 460 89904-50L00·50L01 433MHz P1 98)</t>
         </is>
       </c>
       <c r="P98" s="9" t="inlineStr"/>
@@ -7298,7 +7326,11 @@
         </is>
       </c>
       <c r="K99" s="9" t="inlineStr"/>
-      <c r="L99" s="9" t="inlineStr"/>
+      <c r="L99" s="9" t="inlineStr">
+        <is>
+          <t>89904-50L00[해외 공용 품번], 89904-50L01[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="M99" s="9" t="inlineStr"/>
       <c r="N99" s="9" t="inlineStr">
         <is>
@@ -7307,7 +7339,7 @@
       </c>
       <c r="O99" s="9" t="inlineStr">
         <is>
-          <t>transpondery(LS 460·600h 2009–2012 Texas G DST80 — 433MHz 품번 자료 없음)</t>
+          <t>transpondery(LS 460·600h 2009–2012 Texas G DST80), auto-keys.eu(순정 LS 460 89904-50L00·50L01 433MHz P1 98)</t>
         </is>
       </c>
       <c r="P99" s="9" t="inlineStr"/>
@@ -7364,7 +7396,11 @@
         </is>
       </c>
       <c r="K100" s="9" t="inlineStr"/>
-      <c r="L100" s="9" t="inlineStr"/>
+      <c r="L100" s="9" t="inlineStr">
+        <is>
+          <t>89904-50L00[해외 공용 품번], 89904-50L01[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="M100" s="9" t="inlineStr"/>
       <c r="N100" s="9" t="inlineStr">
         <is>
@@ -7373,7 +7409,7 @@
       </c>
       <c r="O100" s="9" t="inlineStr">
         <is>
-          <t>transpondery(LS 460·600h 2009–2012 Texas G DST80 — 433MHz 품번 자료 없음)</t>
+          <t>transpondery(LS 460·600h 2009–2012 Texas G DST80), auto-keys.eu(순정 LS 460 89904-50L00·50L01 433MHz P1 98)</t>
         </is>
       </c>
       <c r="P100" s="9" t="inlineStr"/>
@@ -7430,7 +7466,11 @@
         </is>
       </c>
       <c r="K101" s="9" t="inlineStr"/>
-      <c r="L101" s="9" t="inlineStr"/>
+      <c r="L101" s="9" t="inlineStr">
+        <is>
+          <t>89904-50L00[해외 공용 품번], 89904-50L01[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="M101" s="9" t="inlineStr"/>
       <c r="N101" s="9" t="inlineStr">
         <is>
@@ -7439,7 +7479,7 @@
       </c>
       <c r="O101" s="9" t="inlineStr">
         <is>
-          <t>transpondery(LS 460·600h 2013–2017 Texas G DST80, 비상키 69515-30380 — 433MHz 품번 자료 없음)</t>
+          <t>transpondery(LS 460·600h 2013–2017 Texas G DST80, 비상키 69515-30380), auto-keys.eu(LS 460 89904-50L00·50L01 433MHz P1 98)</t>
         </is>
       </c>
       <c r="P101" s="9" t="inlineStr"/>
@@ -7496,7 +7536,11 @@
         </is>
       </c>
       <c r="K102" s="9" t="inlineStr"/>
-      <c r="L102" s="9" t="inlineStr"/>
+      <c r="L102" s="9" t="inlineStr">
+        <is>
+          <t>89904-50L00[해외 공용 품번], 89904-50L01[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="M102" s="9" t="inlineStr"/>
       <c r="N102" s="9" t="inlineStr">
         <is>
@@ -7505,7 +7549,7 @@
       </c>
       <c r="O102" s="9" t="inlineStr">
         <is>
-          <t>transpondery(LS 460·600h 2013–2017 Texas G DST80, 비상키 69515-30380 — 433MHz 품번 자료 없음)</t>
+          <t>transpondery(LS 460·600h 2013–2017 Texas G DST80, 비상키 69515-30380), auto-keys.eu(LS 460 89904-50L00·50L01 433MHz P1 98)</t>
         </is>
       </c>
       <c r="P102" s="9" t="inlineStr"/>
@@ -7562,7 +7606,11 @@
         </is>
       </c>
       <c r="K103" s="9" t="inlineStr"/>
-      <c r="L103" s="9" t="inlineStr"/>
+      <c r="L103" s="9" t="inlineStr">
+        <is>
+          <t>89904-50L00[해외 공용 품번], 89904-50L01[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="M103" s="9" t="inlineStr"/>
       <c r="N103" s="9" t="inlineStr">
         <is>
@@ -7571,7 +7619,7 @@
       </c>
       <c r="O103" s="9" t="inlineStr">
         <is>
-          <t>transpondery(LS 460·600h 2013–2017 Texas G DST80, 비상키 69515-30380 — 433MHz 품번 자료 없음)</t>
+          <t>transpondery(LS 460·600h 2013–2017 Texas G DST80, 비상키 69515-30380), auto-keys.eu(LS 460 89904-50L00·50L01 433MHz P1 98)</t>
         </is>
       </c>
       <c r="P103" s="9" t="inlineStr"/>
@@ -7628,7 +7676,11 @@
         </is>
       </c>
       <c r="K104" s="9" t="inlineStr"/>
-      <c r="L104" s="9" t="inlineStr"/>
+      <c r="L104" s="9" t="inlineStr">
+        <is>
+          <t>89904-50L00[해외 공용 품번], 89904-50L01[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="M104" s="9" t="inlineStr"/>
       <c r="N104" s="9" t="inlineStr">
         <is>
@@ -7637,7 +7689,7 @@
       </c>
       <c r="O104" s="9" t="inlineStr">
         <is>
-          <t>transpondery(LS 460·600h 2013–2017 Texas G DST80, 비상키 69515-30380 — 433MHz 품번 자료 없음)</t>
+          <t>transpondery(LS 460·600h 2013–2017 Texas G DST80, 비상키 69515-30380), auto-keys.eu(LS 460 89904-50L00·50L01 433MHz P1 98)</t>
         </is>
       </c>
       <c r="P104" s="9" t="inlineStr"/>
@@ -7694,7 +7746,11 @@
         </is>
       </c>
       <c r="K105" s="9" t="inlineStr"/>
-      <c r="L105" s="9" t="inlineStr"/>
+      <c r="L105" s="9" t="inlineStr">
+        <is>
+          <t>89904-50L00[해외 공용 품번], 89904-50L01[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="M105" s="9" t="inlineStr"/>
       <c r="N105" s="9" t="inlineStr">
         <is>
@@ -7703,7 +7759,7 @@
       </c>
       <c r="O105" s="9" t="inlineStr">
         <is>
-          <t>transpondery(LS 460·600h 2013–2017 Texas G DST80, 비상키 69515-30380 — 433MHz 품번 자료 없음)</t>
+          <t>transpondery(LS 460·600h 2013–2017 Texas G DST80, 비상키 69515-30380), auto-keys.eu(LS 460 89904-50L00·50L01 433MHz P1 98)</t>
         </is>
       </c>
       <c r="P105" s="9" t="inlineStr"/>
@@ -12574,7 +12630,7 @@
       <c r="K178" s="9" t="inlineStr"/>
       <c r="L178" s="9" t="inlineStr">
         <is>
-          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
+          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48244[해외 공용 품번], 89904-48245[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M178" s="9" t="inlineStr"/>
@@ -12644,7 +12700,7 @@
       <c r="K179" s="9" t="inlineStr"/>
       <c r="L179" s="9" t="inlineStr">
         <is>
-          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
+          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48244[해외 공용 품번], 89904-48245[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M179" s="9" t="inlineStr"/>
@@ -12714,7 +12770,7 @@
       <c r="K180" s="9" t="inlineStr"/>
       <c r="L180" s="9" t="inlineStr">
         <is>
-          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
+          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48244[해외 공용 품번], 89904-48245[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M180" s="9" t="inlineStr"/>
@@ -12784,7 +12840,7 @@
       <c r="K181" s="9" t="inlineStr"/>
       <c r="L181" s="9" t="inlineStr">
         <is>
-          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
+          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48244[해외 공용 품번], 89904-48245[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M181" s="9" t="inlineStr"/>
@@ -12854,7 +12910,7 @@
       <c r="K182" s="9" t="inlineStr"/>
       <c r="L182" s="9" t="inlineStr">
         <is>
-          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
+          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48244[해외 공용 품번], 89904-48245[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M182" s="9" t="inlineStr"/>
@@ -12924,7 +12980,7 @@
       <c r="K183" s="9" t="inlineStr"/>
       <c r="L183" s="9" t="inlineStr">
         <is>
-          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
+          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48244[해외 공용 품번], 89904-48245[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M183" s="9" t="inlineStr"/>
@@ -12994,7 +13050,7 @@
       <c r="K184" s="9" t="inlineStr"/>
       <c r="L184" s="9" t="inlineStr">
         <is>
-          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
+          <t>89904-48242[해외 공용 품번], 89904-48243[해외 공용 품번], 89904-48244[해외 공용 품번], 89904-48245[해외 공용 품번], 89904-48521[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M184" s="9" t="inlineStr"/>

</xml_diff>